<commit_message>
update new line for tuto
</commit_message>
<xml_diff>
--- a/outline_keys.xlsx
+++ b/outline_keys.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="150">
   <si>
     <t xml:space="preserve">Port</t>
   </si>
@@ -29,15 +29,6 @@
   </si>
   <si>
     <t xml:space="preserve">Key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8381</t>
-  </si>
-  <si>
-    <t xml:space="preserve">foobar1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ss://Y2hhY2hhMjAtaWV0Zi1wb2x5MTMwNTpmb29iYXIx@ss.quickaccessmm.shop:8381</t>
   </si>
   <si>
     <t xml:space="preserve">8382</t>
@@ -846,554 +837,543 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>20</v>
+        <v>16</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>41</v>
+        <v>37</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>44</v>
+        <v>40</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>50</v>
+        <v>46</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>53</v>
+        <v>49</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>65</v>
+        <v>61</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="2" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="2" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>